<commit_message>
docus and customer flow fixed
</commit_message>
<xml_diff>
--- a/newtax_leads_sample_20.xlsx
+++ b/newtax_leads_sample_20.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDF13FB-FAE3-4554-8CEE-353DF90BEB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Tax Leads TY2025" state="visible" r:id="rId4"/>
+    <sheet name="Tax Leads TY2025" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -886,25 +890,25 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Poppins"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Poppins"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1E293B"/>
-      <sz val="10"/>
       <name val="Poppins"/>
     </font>
   </fonts>
@@ -1317,9 +1321,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -1327,8 +1331,8 @@
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
+    <col min="8" max="8" width="42" customWidth="1"/>
     <col min="9" max="9" width="24" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
@@ -1341,7 +1345,7 @@
     <col min="18" max="18" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1397,7 +1401,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -1453,7 +1457,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>35</v>
       </c>
@@ -1509,7 +1513,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>50</v>
       </c>
@@ -1565,7 +1569,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>66</v>
       </c>
@@ -1621,7 +1625,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>81</v>
       </c>
@@ -1677,7 +1681,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>95</v>
       </c>
@@ -1733,7 +1737,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>108</v>
       </c>
@@ -1789,7 +1793,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>122</v>
       </c>
@@ -1845,7 +1849,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>135</v>
       </c>
@@ -1901,7 +1905,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>148</v>
       </c>
@@ -1957,7 +1961,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>161</v>
       </c>
@@ -2013,7 +2017,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>173</v>
       </c>
@@ -2069,7 +2073,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>188</v>
       </c>
@@ -2125,7 +2129,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>201</v>
       </c>
@@ -2181,7 +2185,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>214</v>
       </c>
@@ -2237,7 +2241,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>228</v>
       </c>
@@ -2293,7 +2297,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>240</v>
       </c>
@@ -2349,7 +2353,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>253</v>
       </c>
@@ -2405,7 +2409,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>265</v>
       </c>
@@ -2461,7 +2465,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>277</v>
       </c>
@@ -2519,6 +2523,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>